<commit_message>
feat: TC-PCS-031/032 -- full 3-intermediary chain LI->HK
Two new pacs.008 testcases exercising the maximum CBPR+ intermediary
agent chain (3 hops), with EUR payments from Liechtenstein to
Hong Kong:

TC-PCS-031: LI(LGT Vaduz) -> CH(UBS Zurich) -> DE(Deutsche Bank
  FFM) -> UK(HSBC London) -> HK(HSBC HK)
  EUR 250'000, ChrgBr=SHAR, investment allocation

TC-PCS-032: LI(LGT Vaduz) -> CH(UBS Zurich) -> DE(Deutsche Bank
  FFM) -> SG(Standard Chartered Singapore) -> HK(HSBC HK)
  EUR 175'000, ChrgBr=SHAR, commodity settlement, alternative
  Asia-Pacific routing via Singapore

Both testcases use all three IntrmyAgt slots (IntrmyAgt1/2/3) with
real-world BICs. Previously the maximum was 2 intermediaries
(TC-PCS-012). CBPR+ pacs.008.001.08 supports up to 3.

examples/pacs.008/ regenerated with 53 XMLs.

Acceptance: pytest 802 passed, pacs.008 53/53 pass.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/testfaelle_pacs008_comprehensive.xlsx
+++ b/templates/testfaelle_pacs008_comprehensive.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV52"/>
+  <dimension ref="A1:AV54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9167,6 +9167,370 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TC-PCS-031</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>CBPR+ EUR LI-&gt;HK mit 3 Intermediaries (Maximum)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Maximale Intermediary-Kette: LI-&gt;CH-&gt;DE-&gt;UK-&gt;HK</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>BLFLLI2XXXX</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>HSBCHKHHXXX</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>BLFLLI2XXXX</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>HSBCHKHHXXX</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Vermoegensverwaltung Vaduz AG</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Herrengasse</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>9490</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Vaduz</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>LI2108800000023456789</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>BLFLLI2XXXX</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>UBSWCHZH80A</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>DEUTDEFFXXX</t>
+        </is>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>HBUKGB4BXXX</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>Asia Pacific Trading Ltd</t>
+        </is>
+      </c>
+      <c r="Z53" t="inlineStr">
+        <is>
+          <t>Connaught Road Central</t>
+        </is>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>999077</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>400123456789</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>BBAN</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr">
+        <is>
+          <t>HSBCHKHHXXX</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>250000.00</t>
+        </is>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>INDA</t>
+        </is>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>SHAR</t>
+        </is>
+      </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>Investment allocation Asia Q2 2026</t>
+        </is>
+      </c>
+      <c r="AV53" t="inlineStr">
+        <is>
+          <t>Maximale 3-Intermediary-Chain: LI(LGT)-&gt;CH(UBS)-&gt;DE(DB)-&gt;UK(HSBC LDN)-&gt;HK(HSBC HK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TC-PCS-032</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>CBPR+ EUR LI-&gt;HK, 3 Intermediaries via CH+DE+SG</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Maximale 3-Intermediary-Chain LI-&gt;CH-&gt;DE-&gt;SG-&gt;HK (alle via BIC)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>CBPR+</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>BLFLLI2XXXX</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>HSBCHKHHXXX</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>BLFLLI2XXXX</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>HSBCHKHHXXX</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Stiftung Liechtenstein</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Staedtle</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>9490</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Vaduz</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>LI2108800000023456789</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>BLFLLI2XXXX</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>UBSWCHZH80A</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>DEUTDEFFXXX</t>
+        </is>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>SCBLSGSGXXX</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>HK Commodities Corp</t>
+        </is>
+      </c>
+      <c r="Z54" t="inlineStr">
+        <is>
+          <t>Queens Road</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr">
+        <is>
+          <t>999077</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>400987654321</t>
+        </is>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>BBAN</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr">
+        <is>
+          <t>HSBCHKHHXXX</t>
+        </is>
+      </c>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>175000.00</t>
+        </is>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>INDA</t>
+        </is>
+      </c>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>SHAR</t>
+        </is>
+      </c>
+      <c r="AR54" t="inlineStr">
+        <is>
+          <t>Commodity settlement HK Q2</t>
+        </is>
+      </c>
+      <c r="AV54" t="inlineStr">
+        <is>
+          <t>3-Intermediary-Chain via CH(UBS)-&gt;DE(DB)-&gt;SG(StanChart)-&gt;HK(HSBC)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>